<commit_message>
Add stewardship model, playbook, and structured RACI workbook
</commit_message>
<xml_diff>
--- a/02_roles_and_stewardship/raci-matrix.xlsx
+++ b/02_roles_and_stewardship/raci-matrix.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\GitHub\enterprise-data-governance-operating-system\02_roles_and_stewardship\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF21C5A0-24C3-4C0C-A504-CB754B1132C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2851606F-34E8-44E5-A62B-FBE1B191221B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{1AD25CD0-EE2E-40A9-B489-45C421A1DF9C}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" activeTab="1" xr2:uid="{1AD25CD0-EE2E-40A9-B489-45C421A1DF9C}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="RACI Matrix" sheetId="2" r:id="rId2"/>
     <sheet name="Roles" sheetId="1" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'RACI Matrix'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Roles!$A$1:$F$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,11 +42,278 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="82">
+  <si>
+    <t>RACI Matrix Workbook</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Defines governance activities and maps responsibility across core governance roles.</t>
+  </si>
+  <si>
+    <t>How to use</t>
+  </si>
+  <si>
+    <t>Review each activity, confirm role design, and adjust RACI assignments to match the target operating model.</t>
+  </si>
+  <si>
+    <t>RACI meanings</t>
+  </si>
+  <si>
+    <t>R = Responsible, A = Accountable, C = Consulted, I = Informed</t>
+  </si>
+  <si>
+    <t>Governance rule</t>
+  </si>
+  <si>
+    <t>Each activity should have one clear A, at least one R where execution exists, and limited use of C to avoid ambiguity.</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Role Type</t>
+  </si>
+  <si>
+    <t>Primary Purpose</t>
+  </si>
+  <si>
+    <t>Typical Decisions</t>
+  </si>
+  <si>
+    <t>Typical Activities</t>
+  </si>
+  <si>
+    <t>Escalation Role</t>
+  </si>
+  <si>
+    <t>Executive Sponsor</t>
+  </si>
+  <si>
+    <t>Oversight</t>
+  </si>
+  <si>
+    <t>Provides strategic sponsorship and senior escalation support</t>
+  </si>
+  <si>
+    <t>Approve direction and risk decisions</t>
+  </si>
+  <si>
+    <t>Review KPI and maturity status</t>
+  </si>
+  <si>
+    <t>Final escalation</t>
+  </si>
+  <si>
+    <t>Governance Lead</t>
+  </si>
+  <si>
+    <t>Coordination</t>
+  </si>
+  <si>
+    <t>Designs and coordinates the governance operating model</t>
+  </si>
+  <si>
+    <t>Set standards and facilitate cross-domain decisions</t>
+  </si>
+  <si>
+    <t>Run forums and monitor implementation</t>
+  </si>
+  <si>
+    <t>Level 3 escalation</t>
+  </si>
+  <si>
+    <t>Data Owner</t>
+  </si>
+  <si>
+    <t>Accountability</t>
+  </si>
+  <si>
+    <t>Owns business decisions for a domain or critical asset</t>
+  </si>
+  <si>
+    <t>Approve definitions, thresholds, and sensitive access</t>
+  </si>
+  <si>
+    <t>Resolve disputes and sponsor remediation</t>
+  </si>
+  <si>
+    <t>Level 2 escalation</t>
+  </si>
+  <si>
+    <t>Data Steward</t>
+  </si>
+  <si>
+    <t>Stewardship</t>
+  </si>
+  <si>
+    <t>Coordinates day-to-day governance operations</t>
+  </si>
+  <si>
+    <t>Prioritize issues and maintain artifact quality</t>
+  </si>
+  <si>
+    <t>Track metadata, issues, and changes</t>
+  </si>
+  <si>
+    <t>Level 1 escalation</t>
+  </si>
+  <si>
+    <t>Control Owner</t>
+  </si>
+  <si>
+    <t>Control Execution</t>
+  </si>
+  <si>
+    <t>Executes a specific governance control</t>
+  </si>
+  <si>
+    <t>Confirm control outcome and evidence</t>
+  </si>
+  <si>
+    <t>Run checks and log exceptions</t>
+  </si>
+  <si>
+    <t>Escalates through steward or owner</t>
+  </si>
+  <si>
+    <t>System Owner</t>
+  </si>
+  <si>
+    <t>Enablement</t>
+  </si>
+  <si>
+    <t>Supports technical platform administration and feasibility</t>
+  </si>
+  <si>
+    <t>Advise on implementation constraints</t>
+  </si>
+  <si>
+    <t>Provision access and support system-side changes</t>
+  </si>
+  <si>
+    <t>Technical escalation input</t>
+  </si>
+  <si>
+    <t>Governance Activity</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Approve governance structure</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>Executive oversight with governance lead coordination</t>
+  </si>
+  <si>
+    <t>Approve domain ownership</t>
+  </si>
+  <si>
+    <t>Owner accountability should be explicit</t>
+  </si>
+  <si>
+    <t>Maintain glossary terms</t>
+  </si>
+  <si>
+    <t>Steward maintains, owner approves</t>
+  </si>
+  <si>
+    <t>Define critical data elements</t>
+  </si>
+  <si>
+    <t>Coordinate with reporting and system context</t>
+  </si>
+  <si>
+    <t>Approve DQ thresholds</t>
+  </si>
+  <si>
+    <t>Thresholds tied to business tolerance</t>
+  </si>
+  <si>
+    <t>Execute recurring DQ checks</t>
+  </si>
+  <si>
+    <t>A/R</t>
+  </si>
+  <si>
+    <t>Control owner executes evidence-producing checks</t>
+  </si>
+  <si>
+    <t>Triage data issues</t>
+  </si>
+  <si>
+    <t>Steward coordinates, control owner supports</t>
+  </si>
+  <si>
+    <t>Approve sensitive access</t>
+  </si>
+  <si>
+    <t>Risk-based and traceable</t>
+  </si>
+  <si>
+    <t>Provision technical access</t>
+  </si>
+  <si>
+    <t>System owner executes provisioning</t>
+  </si>
+  <si>
+    <t>Assess material change impact</t>
+  </si>
+  <si>
+    <t>Required for downstream-affecting changes</t>
+  </si>
+  <si>
+    <t>Escalate unresolved cross-domain issue</t>
+  </si>
+  <si>
+    <t>Governance lead stabilizes cross-domain escalation</t>
+  </si>
+  <si>
+    <t>Review governance KPI trends</t>
+  </si>
+  <si>
+    <t>Used for oversight and maturity review</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +340,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,27 +658,570 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CBAC363-A388-4734-9A05-432BA301700B}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="93.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="135" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C20C8F3-E386-4823-9CEF-F24CFA5A2F0F}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="31.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.46484375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44.265625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" t="s">
+        <v>57</v>
+      </c>
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H13" xr:uid="{6C20C8F3-E386-4823-9CEF-F24CFA5A2F0F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABFD4BA1-D800-49FE-B46C-A93B4C9EBFB5}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F7" xr:uid="{ABFD4BA1-D800-49FE-B46C-A93B4C9EBFB5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>